<commit_message>
Add Event 2: the 17 Event groups not actually posted in the Mac sleep-interrupted run
A run on the new Mac setup got cut off mid-category when the laptop lid
closed and macOS suspended the Chrome<->chromedriver connection
(invalid session id / DevTools disconnected) -- 11 of 28 Event groups
got a real post, 3 more were attempted but failed once the browser
session had already died, and the remaining 14 were never reached.

Duplicated those 17 (3 failed + 14 untouched) into a new "Event 2"
category, same pattern as Тест/Тест 2 -- the original Event category is
left as-is so the next run can target just the remainder without
reposting to the 11 that already went through.
</commit_message>
<xml_diff>
--- a/Page_Bard/groups.xlsx
+++ b/Page_Bard/groups.xlsx
@@ -117,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -160,6 +160,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -527,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C922"/>
+  <dimension ref="A1:C939"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -15513,7 +15519,295 @@
         </is>
       </c>
     </row>
-    <row r="923" ht="25" customHeight="1"/>
+    <row r="923" ht="25" customHeight="1">
+      <c r="A923" s="20" t="inlineStr">
+        <is>
+          <t>Девочки. Израиль.</t>
+        </is>
+      </c>
+      <c r="B923" s="20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/897192168462907/</t>
+        </is>
+      </c>
+      <c r="C923" s="20" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="20" t="inlineStr">
+        <is>
+          <t>Клуб любителей театра и кино в Израиле</t>
+        </is>
+      </c>
+      <c r="B924" s="20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1084611341608897/</t>
+        </is>
+      </c>
+      <c r="C924" s="20" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="20" t="inlineStr">
+        <is>
+          <t>BILETY.CO.IL – агрегатор билетов на спектакли и концерты в Израиле.</t>
+        </is>
+      </c>
+      <c r="B925" s="20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/weekend.il/</t>
+        </is>
+      </c>
+      <c r="C925" s="20" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="20" t="inlineStr">
+        <is>
+          <t>Израиль-повседневная жизнь.</t>
+        </is>
+      </c>
+      <c r="B926" s="20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1628212920761200/</t>
+        </is>
+      </c>
+      <c r="C926" s="20" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="20" t="inlineStr">
+        <is>
+          <t>Афиша в Израиле 🎯</t>
+        </is>
+      </c>
+      <c r="B927" s="20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/afishail/</t>
+        </is>
+      </c>
+      <c r="C927" s="20" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="20" t="inlineStr">
+        <is>
+          <t>Что и Где, Когда и Как</t>
+        </is>
+      </c>
+      <c r="B928" s="20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1633214516929486/</t>
+        </is>
+      </c>
+      <c r="C928" s="20" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="20" t="inlineStr">
+        <is>
+          <t>Рекомендации (המלצות): на блюдечке с голубой каёмочкой</t>
+        </is>
+      </c>
+      <c r="B929" s="20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/267673493681466/</t>
+        </is>
+      </c>
+      <c r="C929" s="20" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="20" t="inlineStr">
+        <is>
+          <t>Стильные ДевчОнки בנות בסטייל</t>
+        </is>
+      </c>
+      <c r="B930" s="20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1842049746034969/</t>
+        </is>
+      </c>
+      <c r="C930" s="20" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="20" t="inlineStr">
+        <is>
+          <t>Events&amp;Shows Israel</t>
+        </is>
+      </c>
+      <c r="B931" s="20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/2058582517693314/</t>
+        </is>
+      </c>
+      <c r="C931" s="20" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="20" t="inlineStr">
+        <is>
+          <t>Новенькие, вам рады!</t>
+        </is>
+      </c>
+      <c r="B932" s="20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1563295877305603/</t>
+        </is>
+      </c>
+      <c r="C932" s="20" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="21" t="inlineStr">
+        <is>
+          <t>Израиль - отдыхающий !!!</t>
+        </is>
+      </c>
+      <c r="B933" s="21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/377680662301500</t>
+        </is>
+      </c>
+      <c r="C933" s="21" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="21" t="inlineStr">
+        <is>
+          <t>Горские евреи в душе</t>
+        </is>
+      </c>
+      <c r="B934" s="21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/855081021528572</t>
+        </is>
+      </c>
+      <c r="C934" s="21" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="21" t="inlineStr">
+        <is>
+          <t>Потому, что Девочки🧡Израиль</t>
+        </is>
+      </c>
+      <c r="B935" s="21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/Devochky</t>
+        </is>
+      </c>
+      <c r="C935" s="21" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="21" t="inlineStr">
+        <is>
+          <t>Горские Евреи В Душе❤️ קווקזים ב נשמה</t>
+        </is>
+      </c>
+      <c r="B936" s="21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1002220399830433</t>
+        </is>
+      </c>
+      <c r="C936" s="21" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="21" t="inlineStr">
+        <is>
+          <t>Горские Евреи всего мира❤️</t>
+        </is>
+      </c>
+      <c r="B937" s="21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/2457430481025501</t>
+        </is>
+      </c>
+      <c r="C937" s="21" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="21" t="inlineStr">
+        <is>
+          <t>Куда бы деться на Софаш</t>
+        </is>
+      </c>
+      <c r="B938" s="21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/sofash</t>
+        </is>
+      </c>
+      <c r="C938" s="21" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="21" t="inlineStr">
+        <is>
+          <t>Афиша ᕗ весь Израиль ᕗ Лучшие мероприятия 🇮🇱</t>
+        </is>
+      </c>
+      <c r="B939" s="21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/955602182622769</t>
+        </is>
+      </c>
+      <c r="C939" s="21" t="inlineStr">
+        <is>
+          <t>Event 2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 16 new Alicante/Spain groups to Page_Bard/groups.xlsx
Extracted from the user's bulk groups export (bard_groups_14.csv),
filtered for Alicante name matches, deduplicated against groups already
in the sheet. 15 went into the existing "Аликанте" category; one
country-wide group ("Объявления Испания: Барселона, Валенсия, Аликанте,
Торревьеха, Малага.") went into the existing "Испания" category instead,
per the user's own call -- it isn't specific to Alicante, same
precedent as the earlier Beer Sheva multi-city handling.
</commit_message>
<xml_diff>
--- a/Page_Bard/groups.xlsx
+++ b/Page_Bard/groups.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C984"/>
+  <dimension ref="A1:C1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -16576,6 +16576,278 @@
         </is>
       </c>
     </row>
+    <row r="985">
+      <c r="A985" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте Работа Знакомства Обьявления</t>
+        </is>
+      </c>
+      <c r="B985" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1247083042126031/</t>
+        </is>
+      </c>
+      <c r="C985" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" s="22" t="inlineStr">
+        <is>
+          <t>Солнечный Аликанте/ Sunny Alicante</t>
+        </is>
+      </c>
+      <c r="B986" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/395426747211233/</t>
+        </is>
+      </c>
+      <c r="C986" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" s="22" t="inlineStr">
+        <is>
+          <t>Мир Аликанте • Alicante</t>
+        </is>
+      </c>
+      <c r="B987" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1396258483817388/</t>
+        </is>
+      </c>
+      <c r="C987" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте услуги</t>
+        </is>
+      </c>
+      <c r="B988" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/793464015014372/</t>
+        </is>
+      </c>
+      <c r="C988" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте 📢 ОБЪЯВЛЕНИЯ</t>
+        </is>
+      </c>
+      <c r="B989" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1862983711177404/</t>
+        </is>
+      </c>
+      <c r="C989" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="22" t="inlineStr">
+        <is>
+          <t>Объявления Испания: Барселона, Валенсия, Аликанте, Торревьеха, Малага.</t>
+        </is>
+      </c>
+      <c r="B990" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/949331247070892/</t>
+        </is>
+      </c>
+      <c r="C990" s="22" t="inlineStr">
+        <is>
+          <t>Испания</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="22" t="inlineStr">
+        <is>
+          <t>Реклама Аликанте</t>
+        </is>
+      </c>
+      <c r="B991" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/121793429936458/</t>
+        </is>
+      </c>
+      <c r="C991" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте - сказочный отдых!</t>
+        </is>
+      </c>
+      <c r="B992" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1531118960439297/</t>
+        </is>
+      </c>
+      <c r="C992" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="22" t="inlineStr">
+        <is>
+          <t>Испания Аликанте Барахолка</t>
+        </is>
+      </c>
+      <c r="B993" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/341797922845430/</t>
+        </is>
+      </c>
+      <c r="C993" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте Сегодня - новостной портал Аликанте на русском языке</t>
+        </is>
+      </c>
+      <c r="B994" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/alicantetoday/</t>
+        </is>
+      </c>
+      <c r="C994" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="22" t="inlineStr">
+        <is>
+          <t>Испания, Аликанте - Продаю/Покупаю.</t>
+        </is>
+      </c>
+      <c r="B995" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/565600561023455/</t>
+        </is>
+      </c>
+      <c r="C995" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="22" t="inlineStr">
+        <is>
+          <t>Мамы и папы в Аликанте</t>
+        </is>
+      </c>
+      <c r="B996" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/229346674147778/</t>
+        </is>
+      </c>
+      <c r="C996" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="22" t="inlineStr">
+        <is>
+          <t>Торревьеха Аликанте Гвардемар Дения Алтея По русски👍🏼</t>
+        </is>
+      </c>
+      <c r="B997" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/679334608836265/</t>
+        </is>
+      </c>
+      <c r="C997" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="22" t="inlineStr">
+        <is>
+          <t>Услуги и работа в Аликанте. Русскоязычная группа.</t>
+        </is>
+      </c>
+      <c r="B998" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/6769236433195039/</t>
+        </is>
+      </c>
+      <c r="C998" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="22" t="inlineStr">
+        <is>
+          <t>ОБЪЯВЛЕНИЯ ‼️‼️‼️ АЛИКАНТЕ - БЕНИДОРМ- ВАЛЕНСИЯ ‼️‼️‼️</t>
+        </is>
+      </c>
+      <c r="B999" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/625627860270677/</t>
+        </is>
+      </c>
+      <c r="C999" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="22" t="inlineStr">
+        <is>
+          <t>Услуги в Аликанте</t>
+        </is>
+      </c>
+      <c r="B1000" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/461064077415596/</t>
+        </is>
+      </c>
+      <c r="C1000" s="22" t="inlineStr">
+        <is>
+          <t>Аликанте</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 2 confirmed-bad London groups as Error_NoPostField
Both failed Error_NoPostField in a live run:
- [londontheatrereview] (likely a corrupted duplicate of the existing
  #КакМнеТеатрвЛондоне row, same URL slug minus a trailing "uk")
- МЫ в Лондоне / UK

"Доска Объявлений в Лондоне" also failed but with a generic Error
(timeout), not Error_NoPostField -- left alone per convention, a single
transient failure isn't treated as confirmed-bad.
</commit_message>
<xml_diff>
--- a/Page_Bard/groups.xlsx
+++ b/Page_Bard/groups.xlsx
@@ -11349,7 +11349,7 @@
       </c>
       <c r="C665" s="12" t="inlineStr">
         <is>
-          <t>Лондон</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -12114,7 +12114,7 @@
       </c>
       <c r="C710" s="12" t="inlineStr">
         <is>
-          <t>Лондон</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 24 new London/England groups to a new "Лондон 2" category
Took 5 export attempts (3 CSV exports via the group-export flow, 2
direct console scrapes) before one finally captured the user's recently
joined batch -- the first several each came back with zero new
London/England matches despite containing the existing 21/23 already in
the sheet, suggesting the earlier exports just hadn't scrolled far
enough to reach the newest joins. This one found 17 London + 7
England/Britain groups not already present.

Per the user's own instruction, kept separate from the existing
"Лондон" category (23 groups) rather than merged into it, and any
"Англия"-named group routed here too.
</commit_message>
<xml_diff>
--- a/Page_Bard/groups.xlsx
+++ b/Page_Bard/groups.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1019"/>
+  <dimension ref="A1:C1043"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -17171,6 +17171,414 @@
         </is>
       </c>
     </row>
+    <row r="1020">
+      <c r="A1020" s="22" t="inlineStr">
+        <is>
+          <t>БГ-ХЕЛП ЛОНДОН</t>
+        </is>
+      </c>
+      <c r="B1020" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/126675055939723/</t>
+        </is>
+      </c>
+      <c r="C1020" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="22" t="inlineStr">
+        <is>
+          <t>АНГЛИЯ | Новости, oбъявления, работа, жилье в Лондоне</t>
+        </is>
+      </c>
+      <c r="B1021" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/england.news.advert.job.house.rent/</t>
+        </is>
+      </c>
+      <c r="C1021" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="22" t="inlineStr">
+        <is>
+          <t>обяви Лондон</t>
+        </is>
+      </c>
+      <c r="B1022" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1671258022904963/</t>
+        </is>
+      </c>
+      <c r="C1022" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="22" t="inlineStr">
+        <is>
+          <t>ЛОНДОН- БГ ХЕЛП</t>
+        </is>
+      </c>
+      <c r="B1023" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/398299661461105/</t>
+        </is>
+      </c>
+      <c r="C1023" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="22" t="inlineStr">
+        <is>
+          <t>Обяви Лондон</t>
+        </is>
+      </c>
+      <c r="B1024" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1009099949205524/</t>
+        </is>
+      </c>
+      <c r="C1024" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="22" t="inlineStr">
+        <is>
+          <t>Наши в Лондоне - Робота Жилье Услуги</t>
+        </is>
+      </c>
+      <c r="B1025" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/244847707906981/</t>
+        </is>
+      </c>
+      <c r="C1025" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="22" t="inlineStr">
+        <is>
+          <t>Обяви Лондон</t>
+        </is>
+      </c>
+      <c r="B1026" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/obiavilondon/</t>
+        </is>
+      </c>
+      <c r="C1026" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="22" t="inlineStr">
+        <is>
+          <t>Лондон по-нашому, Англія (Ukrainians, London, England)</t>
+        </is>
+      </c>
+      <c r="B1027" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/londonponashomu/</t>
+        </is>
+      </c>
+      <c r="C1027" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="22" t="inlineStr">
+        <is>
+          <t>Лондон</t>
+        </is>
+      </c>
+      <c r="B1028" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/158762847623967/</t>
+        </is>
+      </c>
+      <c r="C1028" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="22" t="inlineStr">
+        <is>
+          <t>Лондон - Англія - Оголошення</t>
+        </is>
+      </c>
+      <c r="B1029" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/5992024727546127/</t>
+        </is>
+      </c>
+      <c r="C1029" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="22" t="inlineStr">
+        <is>
+          <t>Доска Объявлений Лондон</t>
+        </is>
+      </c>
+      <c r="B1030" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/2424938907835471/</t>
+        </is>
+      </c>
+      <c r="C1030" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="22" t="inlineStr">
+        <is>
+          <t>Русскоговорящие в London ( Russian speakers in London )</t>
+        </is>
+      </c>
+      <c r="B1031" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1534976066768785/</t>
+        </is>
+      </c>
+      <c r="C1031" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="22" t="inlineStr">
+        <is>
+          <t>Russians in London | Русские в Лондоне</t>
+        </is>
+      </c>
+      <c r="B1032" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/838970723769036/</t>
+        </is>
+      </c>
+      <c r="C1032" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="22" t="inlineStr">
+        <is>
+          <t>Жизнь Восточного Лондона (East London)</t>
+        </is>
+      </c>
+      <c r="B1033" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/797286882069924/</t>
+        </is>
+      </c>
+      <c r="C1033" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" s="22" t="inlineStr">
+        <is>
+          <t>Наш Лондон 🇬🇧🫶</t>
+        </is>
+      </c>
+      <c r="B1034" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/450560866744845/</t>
+        </is>
+      </c>
+      <c r="C1034" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="22" t="inlineStr">
+        <is>
+          <t>Русские мамы в Лондоне</t>
+        </is>
+      </c>
+      <c r="B1035" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/316721102820184/</t>
+        </is>
+      </c>
+      <c r="C1035" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="22" t="inlineStr">
+        <is>
+          <t>Лондон-Англия-Объявления</t>
+        </is>
+      </c>
+      <c r="B1036" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1525093397774204/</t>
+        </is>
+      </c>
+      <c r="C1036" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="22" t="inlineStr">
+        <is>
+          <t>Великобритания</t>
+        </is>
+      </c>
+      <c r="B1037" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/RussianBritania/</t>
+        </is>
+      </c>
+      <c r="C1037" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="22" t="inlineStr">
+        <is>
+          <t>Наши в Англии (Great Britain)</t>
+        </is>
+      </c>
+      <c r="B1038" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/nashivanglii/</t>
+        </is>
+      </c>
+      <c r="C1038" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="22" t="inlineStr">
+        <is>
+          <t>Русскоязычные В Англии И Зарубежом</t>
+        </is>
+      </c>
+      <c r="B1039" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1025108274177027/</t>
+        </is>
+      </c>
+      <c r="C1039" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="22" t="inlineStr">
+        <is>
+          <t>Русский Форум в Англии</t>
+        </is>
+      </c>
+      <c r="B1040" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/286834915839554/</t>
+        </is>
+      </c>
+      <c r="C1040" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="22" t="inlineStr">
+        <is>
+          <t>Наши в Великобритании, Англии</t>
+        </is>
+      </c>
+      <c r="B1041" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/233522196227996/</t>
+        </is>
+      </c>
+      <c r="C1041" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" s="22" t="inlineStr">
+        <is>
+          <t>Русскоговорящие в Англии (Russians in England)</t>
+        </is>
+      </c>
+      <c r="B1042" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/RussiaInEngland/</t>
+        </is>
+      </c>
+      <c r="C1042" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="22" t="inlineStr">
+        <is>
+          <t>Доска Объявлений в Англии</t>
+        </is>
+      </c>
+      <c r="B1043" s="22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/199672256779044/</t>
+        </is>
+      </c>
+      <c r="C1043" s="22" t="inlineStr">
+        <is>
+          <t>Лондон 2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 3 confirmed-bad Beer Sheva groups as Error_NoPostField
- Беер шева и всё что с ней связано
- Дорога домой (Беер Шева и негев...) помощь животным
- Иерусалим-Бейт Шемеш-Модиин. Поиск работы Тель авив Ашдод, Беер Шева, Хайфа
</commit_message>
<xml_diff>
--- a/Page_Bard/groups.xlsx
+++ b/Page_Bard/groups.xlsx
@@ -16385,7 +16385,7 @@
       </c>
       <c r="C973" s="22" t="inlineStr">
         <is>
-          <t>Беэр Шева</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -16419,7 +16419,7 @@
       </c>
       <c r="C975" s="22" t="inlineStr">
         <is>
-          <t>Беэр Шева</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -16521,7 +16521,7 @@
       </c>
       <c r="C981" s="22" t="inlineStr">
         <is>
-          <t>Беэр Шева</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>

</xml_diff>